<commit_message>
Update stock data and decimal entry
</commit_message>
<xml_diff>
--- a/lagerbestand_vorlage_mass_schoen.xlsx
+++ b/lagerbestand_vorlage_mass_schoen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nils Wienstroer\Documents\Codex\Projekte\aktiv\Lagerbestell App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80A64799-3805-46F9-BDD6-9B272BCAA866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F0B814-25D0-45B2-AA4C-F6597FE68D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-32168" yWindow="-25" windowWidth="32281" windowHeight="17656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -950,7 +950,7 @@
         <v>26</v>
       </c>
       <c r="C7" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="4" t="s">
@@ -998,7 +998,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="4" t="s">

</xml_diff>